<commit_message>
Recodificación PE041 -> pd03 y etiquetas
</commit_message>
<xml_diff>
--- a/data-raw/xlsx/tabla_pd03.xlsx
+++ b/data-raw/xlsx/tabla_pd03.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ucao365-my.sharepoint.com/personal/fernando_gallegos_uca_edu_ar/Documents/proyectos/2026-03-11 Bases EU-SILC/documentos/tablas/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fernando_gallegos\Proyectos\odsa.eusilc\data-raw\xlsx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="68" documentId="11_AD4D2F04E46CFB4ACB3E20B8E5D4D930683EDF2B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2AA0A635-30A2-4C69-8AEC-5122D675C70A}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4ADD520C-AA4E-4D69-B364-94BD50A3651D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20640" windowHeight="11760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -516,7 +516,7 @@
         <v>400</v>
       </c>
       <c r="B21">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
@@ -524,7 +524,7 @@
         <v>440</v>
       </c>
       <c r="B22">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
@@ -532,7 +532,7 @@
         <v>450</v>
       </c>
       <c r="B23">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
@@ -540,7 +540,7 @@
         <v>490</v>
       </c>
       <c r="B24">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
@@ -580,7 +580,7 @@
         <v>600</v>
       </c>
       <c r="B29">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
@@ -588,7 +588,7 @@
         <v>700</v>
       </c>
       <c r="B30">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
@@ -596,7 +596,7 @@
         <v>800</v>
       </c>
       <c r="B31">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>